<commit_message>
refactor excel_book_finder.py and excel_book_finder_tester.xlsx
</commit_message>
<xml_diff>
--- a/resources/scenarios/excel_book_finder_tester.xlsx
+++ b/resources/scenarios/excel_book_finder_tester.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\finge\PycharmProjects\EbfData\resources\scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9720726D-86DD-4A17-9697-A0C811761E97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8220B69-F8EA-4AA5-B21A-AE6554403BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58560" yWindow="2445" windowWidth="22920" windowHeight="13050" xr2:uid="{E4BC70C9-E300-458D-81B1-A3421511F121}"/>
+    <workbookView xWindow="-27610" yWindow="6900" windowWidth="22920" windowHeight="13050" xr2:uid="{E4BC70C9-E300-458D-81B1-A3421511F121}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="LOCAL_SCOPE" localSheetId="0">Sheet1!$C$9</definedName>
+    <definedName name="MEANING_OF_LIFE">42</definedName>
+    <definedName name="MIN" localSheetId="0">18</definedName>
     <definedName name="WBK_SCOPE">Sheet1!$C$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -66,20 +68,28 @@
     <t>wks scoped name</t>
   </si>
   <si>
-    <t>WKB</t>
-  </si>
-  <si>
-    <t>Sheet1</t>
+    <t>some global value</t>
+  </si>
+  <si>
+    <t>some local value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -93,7 +103,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -101,14 +111,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Explanatory Text" xfId="1" builtinId="53"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -456,7 +485,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="2:4">
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -484,19 +513,21 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="2:4">
-      <c r="C7" t="s">
+    <row r="6" spans="2:4" ht="15" thickBot="1"/>
+    <row r="7" spans="2:4" ht="15" thickBot="1">
+      <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
-      <c r="C9" t="s">
+    <row r="8" spans="2:4" ht="15" thickBot="1"/>
+    <row r="9" spans="2:4" ht="15" thickBot="1">
+      <c r="C9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>